<commit_message>
Fase 9, G12: calibración final y documentación.
Calculadora: la sección "Reglas de pago" revisa también lo que aún no
tiene id ("Próximamente"), con precio y columna Id, ordenada. 18
productos, todos cosméticos o el pase; 14 sin id.

Calibración con todo encendido, sin alertas y sin cambiar números:
el habitual termina el pase el día 23 y gasta el 97 % de su Ámbar; el
casual llega al nivel 13; el intenso, día 13; amigos, día 20. Prueba de
robustez (ritmos ×0,7, sesiones cortas) apuntada como hallazgo en la
skill, con la línea base nueva.

Documentación: GDD v0.3 (§4 misiones v2 y semanales, §5.4 contratos,
eventos y Gran Tropa, §11, §14 pase, tiendas, cosméticos y
correcciones), VERIFICACION §10, LANZAMIENTO (Developer Products a
crear, fecha de la T1, publicar los tres places a la vez) y hoja
"Correcciones" en el Excel del pase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/battle_pass_30_days.xlsx
+++ b/docs/battle_pass_30_days.xlsx
@@ -14,6 +14,7 @@
   </bookViews>
   <sheets>
     <sheet name="Modelo Recompensas 30 Días" sheetId="1" r:id="rId1"/>
+    <sheet name="Correcciones" sheetId="2" r:id="rId99"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2088,4 +2089,899 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="62" customWidth="1"/>
+    <col min="3" max="3" width="62" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correcciones del modelo (21-10-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lo que cambió al pasar este modelo al juego (docs/GDD.md §14.4). Los números de verdad están en src/shared/Config.luau (Season, Daily, Shop) y src/shared/Data/Seasons.luau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. HALLAZGOS 7–10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Este modelo decía</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En el juego</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por qué</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La premium vende aceleradores del nido y Ámbar</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium 100 % cosmética; el Ámbar y el tiempo de huevo solo en la pista gratis</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El Ámbar compra mejoras de vida y daño: venderlo es pagar para ganar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Superviviente de la Isla" en el nivel 30 gratis</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El N30 gratis da el título "Señor del Volcán"</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Superviviente" es solo para quien gana una partida</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skins de Tití, Mandril y Gorila Albino; total premium 90 (suma 75); 1.000 XP al día justos</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skins solo de las 13 mascotas reales (y de familia); 30 premios premium, uno por nivel; se termina con ~20–24 días activos</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esos monos no son mascotas; con la XP justa había que jugar los 30 días</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Niveles comprados con sus premios gratis</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los premios no cosméticos solo con nivel ganado jugando</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si no, los niveles de Robux venderían Ámbar y tiempo de huevo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. PARÁMETROS REALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parámetro</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dónde</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duración de la temporada</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 días + 7 de descanso</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.Days / RestDays</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Niveles × XP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 × 1.000 (en bucle: cada 1.500)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.Levels / LevelXp / LoopXp</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Última semana</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×2 de XP</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.LastWeekMultiplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XP de la Isla</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60/día, 150/jefe, 50/huevo, 300/rescate</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.IslandXp</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XP de Dunas</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80 / 40 / 30 + 15 por captura</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.ArenaXp</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tope de partidas</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.200 XP al día (misiones fuera)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.DailyMatchXpCap</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Misiones diarias</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fácil 200 · media 200 · difícil 300 XP</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Daily.MissionRewards</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semanales</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 × 500 XP + 500 por las 5</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Daily.MissionRewards / WeeklyBonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amigos</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+10 %</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Season.FriendsBonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precios</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">premium 399 · pack +10 niveles 799 · nivel 79 R$</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config.Shop.Products</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medido (calculadora)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">habitual termina el día 23; casual nivel 13; intenso día 13; amigos día 20</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/island/tools/Economia.luau</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. TEMPORADA 1: EL DESPERTAR DEL VOLCÁN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nivel</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gratis (ganado jugando)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium (solo cosmético)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Náufrago del Volcán</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aura: Llama primal I</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75 Ámbar</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emote: Grito de gorila</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 bananos + 2 vendas</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arma: Maza de Azufre</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−30 min de huevo + Marco de bronce</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Hijo del Volcán</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 Ámbar</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traje: Guardián del Fuego Azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 antorcha + 1 antídoto + Emote: Saludo simio</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Números: Magma</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−30 min de huevo</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arma: Arco de Azufre</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 Ámbar + Arma: Machete de Azufre</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estallido: Erupción</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 super venda</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emote: Danza del fuego</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150 Ámbar</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traje: Acechador del Fuego Azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−45 min de huevo</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estela: Pisada de magma</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 vendas + Skin: Tortuga de Lava</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nido: Volcánico</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100 Ámbar</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arma: Bastón de Azufre</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−45 min de huevo</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Números: Fuego azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estela de ceniza</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aura: Llama primal II</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">125 Ámbar</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estela de fuego azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 kit de reanimación</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emote: Erupción</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−60 min de huevo</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arma: Cerbatana de Azufre</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">125 Ámbar</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Caminante de Ceniza</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">huevo Raro</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traje: Invocador del Fuego Azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 antídotos + 1 super venda</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marco de fuego azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150 Ámbar + Marco de plata</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estallido: Fuego azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−60 min de huevo</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skin: Jaguar de Magma</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 antorchas + 5 bananos</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Domador del Magma</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200 Ámbar</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traje: Sanador del Fuego Azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−60 min de huevo</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Guardián de la Llama Azul</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 kit de reanimación + 2 super vendas</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marco: Obsidiana fundida</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200 Ámbar</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nido: Cráter de azufre</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−90 min de huevo</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Título: Rey de la Isla Primal</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">300 Ámbar + Título: Señor del Volcán</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aura: Llama primal III</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>